<commit_message>
updated the prompt and added effectiveness data
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Run Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Extracted Data'!$A$1:$T$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Extracted Data'!$A$1:$T$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -416,21 +416,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T4"/>
+  <dimension ref="A1:T6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
     <col width="34" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
     <col width="26" customWidth="1" min="7" max="7"/>
     <col width="20" customWidth="1" min="8" max="8"/>
     <col width="50" customWidth="1" min="9" max="9"/>
     <col width="33" customWidth="1" min="10" max="10"/>
-    <col width="51" customWidth="1" min="11" max="11"/>
-    <col width="29" customWidth="1" min="12" max="12"/>
+    <col width="58" customWidth="1" min="11" max="11"/>
+    <col width="37" customWidth="1" min="12" max="12"/>
     <col width="60" customWidth="1" min="13" max="13"/>
     <col width="29" customWidth="1" min="14" max="14"/>
     <col width="29" customWidth="1" min="15" max="15"/>
@@ -602,6 +602,11 @@
           <t>28.04.2025</t>
         </is>
       </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>granted</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -610,56 +615,56 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bikaner distt.</t>
+          <t>Panipat</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Bikaner-II PS</t>
+          <t>400/220 kV Jind(PG) S/s</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>ACME Solar Holdings Limited</t>
+          <t>Panipat Green Hydrogen Private Limited</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>1200003683</t>
-        </is>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>1200003829</t>
+          <t>2200002261</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>190</t>
+          <t>99</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Generator (Solar)</t>
+          <t>Bulk consumer (including Green Hydrogen / Green Ammonia)</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>seeking to connect to ISTS directly</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>01.12.2025</t>
+          <t>25.08.2027</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>14-08-2025</t>
+          <t>17.07.2025</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>Revoked</t>
+          <t>granted</t>
         </is>
       </c>
     </row>
@@ -670,51 +675,181 @@
         </is>
       </c>
       <c r="B4" t="n">
+        <v>7</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Bikaner distt.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Bikaner-II PS</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ACME Solar Holdings Limited</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>1200003683</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>1200003829</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>190</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Generating station(s), including REGS(s), without ESS</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>01.12.2025</t>
+        </is>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>14-08-2025</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Revoked</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>/home/bittu/Desktop/App-connectivity/start/source_1/177185140447Minutes of 43rd CMETS NR meeting held on 12.01.2026_F.pdf</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>8</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Bikaner-II PS</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>M/s ACME Solar Holdings</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>1200003683</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1200003829</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Generator (Solar)</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>31.03.2027</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>12.12.2025</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>31.03.2027</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>granted</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>300</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>/home/bittu/Desktop/App-connectivity/start/source_1/177185140447Minutes of 43rd CMETS NR meeting held on 12.01.2026_F.pdf</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>9</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Mainpuri (PG) S/s</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
         <is>
           <t>Mainpuri (PG)</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>Mainpuri (PG)</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>Indian Railways</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>2200002494</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>50</t>
         </is>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>Bulk consumer seeking to connect to ISTS directly</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>01.12.2025</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>13.10.2025</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T4"/>
+  <autoFilter ref="A1:T6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -740,7 +875,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>2026-04-22T11:26:18</t>
+          <t>2026-04-23T15:34:07</t>
         </is>
       </c>
     </row>
@@ -752,7 +887,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-04-22T11:27:48</t>
+          <t>2026-04-23T15:34:44</t>
         </is>
       </c>
     </row>
@@ -763,7 +898,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>89.89</v>
+        <v>36.44</v>
       </c>
     </row>
     <row r="4">
@@ -813,7 +948,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>